<commit_message>
Update repository files without large pptx
</commit_message>
<xml_diff>
--- a/01.SOMD/01.metadata_structure/02_SOMD_search_eq.xlsx
+++ b/01.SOMD/01.metadata_structure/02_SOMD_search_eq.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cgiar.sharepoint.com/sites/Alliance-AgroecologyKnowledgeHub/Shared Documents/General/Agroecology_Evidence_Hub/01.SOMD/01.metadata_structure/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="432" documentId="8_{3DBE2D00-5402-43EC-822D-A8757C7CA091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA648A69-F019-4B12-B178-C776CC2B8BBA}"/>
+  <xr:revisionPtr revIDLastSave="525" documentId="8_{3DBE2D00-5402-43EC-822D-A8757C7CA091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E660F0AA-4609-40FC-842F-D55F4958CD07}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CF94B49-C55C-417E-8862-D75FC6347405}"/>
+    <workbookView minimized="1" xWindow="3075" yWindow="2835" windowWidth="21600" windowHeight="11175" xr2:uid="{6CF94B49-C55C-417E-8862-D75FC6347405}"/>
   </bookViews>
   <sheets>
     <sheet name="03_SOMD_search_eq" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="114">
   <si>
     <t>search_strategy</t>
   </si>
@@ -67,9 +67,6 @@
     <t>search_date</t>
   </si>
   <si>
-    <t>nb_papers</t>
-  </si>
-  <si>
     <t>source_id</t>
   </si>
   <si>
@@ -92,63 +89,6 @@
   </si>
   <si>
     <t>10.1038/s41597-024-03682-6</t>
-  </si>
-  <si>
-    <t>MA</t>
-  </si>
-  <si>
-    <t>Financial profitability of diversified farming systems: A global meta-analysis.</t>
-  </si>
-  <si>
-    <t>Sanchez, A.C., Kamau, H., Grazioli, F., Jones, S.</t>
-  </si>
-  <si>
-    <t>Ecol. Eco</t>
-  </si>
-  <si>
-    <t>10.1016/j.ecolecon.2022.107595</t>
-  </si>
-  <si>
-    <t>MD</t>
-  </si>
-  <si>
-    <t>Effects of changing farming practices in African agriculture.</t>
-  </si>
-  <si>
-    <r>
-      <t>Rosenstock, T.S., Steward, P., Joshi, N. </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="8"/>
-        <color rgb="FF222222"/>
-        <rFont val="Segoe UI"/>
-        <family val="2"/>
-      </rPr>
-      <t>et al.</t>
-    </r>
-  </si>
-  <si>
-    <t>10.1038/s41597-024-03805-z</t>
-  </si>
-  <si>
-    <t>A global database of diversified farming effects on biodiversity and yield</t>
-  </si>
-  <si>
-    <t>Jones, S.K., Sanchez, A.C., et al.</t>
-  </si>
-  <si>
-    <t>10.1038/s41597-021-01000-y</t>
-  </si>
-  <si>
-    <t>Achieving win-win outcomes for biodiversity and yield through diversified farming</t>
-  </si>
-  <si>
-    <t>Basic and Applied Ecology</t>
-  </si>
-  <si>
-    <t>10.1016/j.baae.2022.12.005</t>
   </si>
   <si>
     <t>Dataset section</t>
@@ -427,12 +367,48 @@
     <t>Authors: "List MFL SP Alliance"
 Keyword: “synthesis” OR “meta-analysis” OR “systematic review” OR “data paper” OR “vote-counting”</t>
   </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>RTE_OA</t>
+  </si>
+  <si>
+    <t>RTE_WOS</t>
+  </si>
+  <si>
+    <t>RTE_OA_26.04.2026</t>
+  </si>
+  <si>
+    <t>RTE_WOS_26.04.2026</t>
+  </si>
+  <si>
+    <t>Schievano et al 2024</t>
+  </si>
+  <si>
+    <t>Research Team Evidence (MFL except alliance)</t>
+  </si>
+  <si>
+    <t>Research Team Evidence (MFL Alliance)</t>
+  </si>
+  <si>
+    <t>Open Alex</t>
+  </si>
+  <si>
+    <t>Web of Science</t>
+  </si>
+  <si>
+    <t>Research Team Evidence (Evidence Hub core)</t>
+  </si>
+  <si>
+    <t>n_records</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -489,10 +465,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
-      <sz val="8"/>
-      <color rgb="FF222222"/>
-      <name val="Segoe UI"/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
     <font>
@@ -500,9 +475,32 @@
       <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -535,18 +533,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor rgb="FFDAF2D0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9"/>
         <bgColor theme="9"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -579,30 +571,10 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF8ED973"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF8ED973"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="thin">
         <color theme="9" tint="0.39997558519241921"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FF8ED973"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -621,7 +593,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -630,42 +602,29 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="7" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="11" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="12" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="11">
     <dxf>
       <font>
         <b/>
@@ -960,23 +919,23 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{82829F27-CA0C-4D60-BB23-180295D9F6ED}" name="_03_SOMD_search_eq" displayName="_03_SOMD_search_eq" ref="A1:L10" totalsRowShown="0" tableBorderDxfId="11">
-  <autoFilter ref="A1:L10" xr:uid="{82829F27-CA0C-4D60-BB23-180295D9F6ED}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{82829F27-CA0C-4D60-BB23-180295D9F6ED}" name="_03_SOMD_search_eq" displayName="_03_SOMD_search_eq" ref="A1:L6" totalsRowShown="0" tableBorderDxfId="10">
+  <autoFilter ref="A1:L6" xr:uid="{82829F27-CA0C-4D60-BB23-180295D9F6ED}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{75F0B827-B07E-4D17-9EE6-998B88894E08}" name="search_strategy" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{75F0B827-B07E-4D17-9EE6-998B88894E08}" name="search_strategy" dataDxfId="9"/>
     <tableColumn id="12" xr3:uid="{D50BAE16-3EEC-4F3A-9879-1EBADD3BD934}" name="ss_type"/>
-    <tableColumn id="7" xr3:uid="{7882ED10-B182-427A-8DC8-89E886C219F2}" name="search_database_title" dataDxfId="9"/>
-    <tableColumn id="8" xr3:uid="{8E80BD2B-21B0-4577-92F4-9878E219FABE}" name="search_database_authors" dataDxfId="8"/>
-    <tableColumn id="9" xr3:uid="{4BD55543-C822-40EE-9ADB-74A1A3F8A7BD}" name="search_database_year" dataDxfId="7"/>
-    <tableColumn id="10" xr3:uid="{9C7DD67D-7240-4A87-8DE2-58212E118815}" name="search_database_journal" dataDxfId="6"/>
-    <tableColumn id="11" xr3:uid="{95D4F1CD-3E6E-4C0D-AA2C-3862CCB8E95A}" name="search_database_doi" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{935D10CB-4A20-402C-84F7-9BA030FB443A}" name="search_equations" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{3C572029-E3D3-4089-B204-131CCCA19147}" name="search_date" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{85B333BE-0EAA-4AB1-AAC0-F05626296905}" name="nb_papers"/>
-    <tableColumn id="6" xr3:uid="{D0C08A4F-920A-4575-8579-5CF892FB05D8}" name="source_id" dataDxfId="2">
+    <tableColumn id="7" xr3:uid="{7882ED10-B182-427A-8DC8-89E886C219F2}" name="search_database_title" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{8E80BD2B-21B0-4577-92F4-9878E219FABE}" name="search_database_authors" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{4BD55543-C822-40EE-9ADB-74A1A3F8A7BD}" name="search_database_year" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{9C7DD67D-7240-4A87-8DE2-58212E118815}" name="search_database_journal" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{95D4F1CD-3E6E-4C0D-AA2C-3862CCB8E95A}" name="search_database_doi" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{935D10CB-4A20-402C-84F7-9BA030FB443A}" name="search_equations" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{3C572029-E3D3-4089-B204-131CCCA19147}" name="search_date" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{85B333BE-0EAA-4AB1-AAC0-F05626296905}" name="n_records"/>
+    <tableColumn id="6" xr3:uid="{D0C08A4F-920A-4575-8579-5CF892FB05D8}" name="source_id" dataDxfId="1">
       <calculatedColumnFormula>_03_SOMD_search_eq[[#This Row],[ss_type]]&amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_authors]],5) &amp; "_" &amp; RIGHT(_03_SOMD_search_eq[[#This Row],[search_database_year]],2) &amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_title]],5) &amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_journal]],2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{C4BF67C1-9B1F-4F4E-9D9A-F99584C29016}" name="nb_papers_after_merging" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{C4BF67C1-9B1F-4F4E-9D9A-F99584C29016}" name="nb_papers_after_merging" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1299,10 +1258,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78503B5C-F673-4768-9E9B-BB0C86AF28D2}">
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="23.85546875" customWidth="1"/>
+    <col min="1" max="1" width="40.28515625" customWidth="1"/>
+    <col min="2" max="2" width="23.85546875" customWidth="1"/>
     <col min="3" max="7" width="30.85546875" customWidth="1"/>
     <col min="8" max="8" width="23.85546875" customWidth="1"/>
     <col min="9" max="9" width="26.140625" customWidth="1"/>
@@ -1315,7 +1275,7 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
@@ -1340,39 +1300,39 @@
         <v>8</v>
       </c>
       <c r="J1" t="s">
+        <v>113</v>
+      </c>
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>10</v>
-      </c>
-      <c r="L1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>14</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>15</v>
       </c>
       <c r="E2" s="4">
         <v>2024</v>
       </c>
       <c r="F2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
       <c r="J2">
         <v>13935</v>
       </c>
@@ -1384,260 +1344,157 @@
         <v>13935</v>
       </c>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:12" ht="15" customHeight="1">
       <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="E3" s="4">
-        <v>2022</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H3" s="8"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="3" t="str">
-        <f>_03_SOMD_search_eq[[#This Row],[ss_type]]&amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_authors]],5) &amp; "_" &amp; RIGHT(_03_SOMD_search_eq[[#This Row],[search_database_year]],2) &amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_title]],5) &amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_journal]],2)</f>
-        <v>MA_Sanch_22_Finan_Ec</v>
-      </c>
-      <c r="L3" s="9">
-        <v>1</v>
-      </c>
+        <v>112</v>
+      </c>
+      <c r="B3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="H3" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="I3" s="19">
+        <v>46138</v>
+      </c>
+      <c r="J3">
+        <v>161</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="L3" s="7"/>
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="E4" s="4">
-        <v>2024</v>
+        <v>112</v>
+      </c>
+      <c r="B4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>100</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G4" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="H4" s="8"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="8"/>
-      <c r="K4" s="3" t="str">
-        <f>_03_SOMD_search_eq[[#This Row],[ss_type]]&amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_authors]],5) &amp; "_" &amp; RIGHT(_03_SOMD_search_eq[[#This Row],[search_database_year]],2) &amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_title]],5) &amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_journal]],2)</f>
-        <v>MD_Rosen_24_Effec_Sc</v>
-      </c>
-      <c r="L4" s="12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D5" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="E5" s="4">
-        <v>2021</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="H5" s="8"/>
-      <c r="I5" s="9"/>
-      <c r="K5" s="3" t="str">
-        <f>_03_SOMD_search_eq[[#This Row],[ss_type]]&amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_authors]],5) &amp; "_" &amp; RIGHT(_03_SOMD_search_eq[[#This Row],[search_database_year]],2) &amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_title]],5) &amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_journal]],2)</f>
-        <v>MD_Jones_21_A glo_Sc</v>
-      </c>
-      <c r="L5" s="12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="D6" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="E6" s="4">
-        <v>2023</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="H6" s="8"/>
-      <c r="I6" s="9"/>
-      <c r="K6" s="3" t="str">
-        <f>_03_SOMD_search_eq[[#This Row],[ss_type]]&amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_authors]],5) &amp; "_" &amp; RIGHT(_03_SOMD_search_eq[[#This Row],[search_database_year]],2) &amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_title]],5) &amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_journal]],2)</f>
-        <v>MA_Jones_23_Achie_Ba</v>
-      </c>
-      <c r="L6" s="12"/>
-    </row>
-    <row r="7" spans="1:12">
-      <c r="A7" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="25" t="s">
+        <v>102</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="I4" s="19">
+        <v>46138</v>
+      </c>
+      <c r="J4">
+        <v>49</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="L4" s="7"/>
+    </row>
+    <row r="5" spans="1:12" s="12" customFormat="1">
+      <c r="A5" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="I7" s="19">
-        <v>46138</v>
-      </c>
-      <c r="J7">
-        <v>161</v>
-      </c>
-      <c r="K7" s="3" t="str">
-        <f>_03_SOMD_search_eq[[#This Row],[ss_type]]&amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_authors]],5) &amp; "_" &amp; RIGHT(_03_SOMD_search_eq[[#This Row],[search_database_year]],2) &amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_title]],5) &amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_journal]],2)</f>
-        <v>_Hub c__Open _</v>
-      </c>
-      <c r="L7" s="12"/>
-    </row>
-    <row r="8" spans="1:12">
-      <c r="A8" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="21"/>
-      <c r="C8" s="24" t="s">
+      <c r="B5" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="G5" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="H5" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="I5" s="16">
+        <v>46145</v>
+      </c>
+      <c r="J5" s="12">
+        <v>5</v>
+      </c>
+      <c r="K5" s="17"/>
+      <c r="L5" s="18"/>
+    </row>
+    <row r="6" spans="1:12" s="12" customFormat="1">
+      <c r="A6" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="D8" s="22" t="s">
-        <v>116</v>
-      </c>
-      <c r="E8" s="22"/>
-      <c r="F8" s="22"/>
-      <c r="G8" s="22"/>
-      <c r="H8" s="23" t="s">
+      <c r="B6" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="C6" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="I8" s="19">
-        <v>46138</v>
-      </c>
-      <c r="J8" s="21">
-        <v>49</v>
-      </c>
-      <c r="K8" s="18" t="str">
-        <f>_03_SOMD_search_eq[[#This Row],[ss_type]]&amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_authors]],5) &amp; "_" &amp; RIGHT(_03_SOMD_search_eq[[#This Row],[search_database_year]],2) &amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_title]],5) &amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_journal]],2)</f>
-        <v>_Hub c__Web o_</v>
-      </c>
-      <c r="L8" s="12"/>
-    </row>
-    <row r="9" spans="1:12">
-      <c r="A9" s="18"/>
-      <c r="B9" s="21"/>
-      <c r="C9" s="24" t="s">
-        <v>111</v>
-      </c>
-      <c r="D9" s="22" t="s">
-        <v>114</v>
-      </c>
-      <c r="E9" s="22"/>
-      <c r="F9" s="22"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="23" t="s">
-        <v>112</v>
-      </c>
-      <c r="I9" s="19">
+      <c r="D6" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="G6" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="H6" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="I6" s="16">
         <v>46145</v>
       </c>
-      <c r="J9" s="21">
-        <v>5</v>
-      </c>
-      <c r="K9" s="18" t="str">
-        <f>_03_SOMD_search_eq[[#This Row],[ss_type]]&amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_authors]],5) &amp; "_" &amp; RIGHT(_03_SOMD_search_eq[[#This Row],[search_database_year]],2) &amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_title]],5) &amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_journal]],2)</f>
-        <v>_MFL e__Open _</v>
-      </c>
-      <c r="L9" s="12"/>
-    </row>
-    <row r="10" spans="1:12">
-      <c r="A10" s="18"/>
-      <c r="B10" s="21"/>
-      <c r="C10" s="24" t="s">
-        <v>113</v>
-      </c>
-      <c r="D10" s="22" t="s">
-        <v>115</v>
-      </c>
-      <c r="E10" s="22"/>
-      <c r="F10" s="22"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="20" t="s">
-        <v>117</v>
-      </c>
-      <c r="I10" s="19">
-        <v>46145</v>
-      </c>
-      <c r="J10" s="21">
+      <c r="J6" s="12">
         <v>691</v>
       </c>
-      <c r="K10" s="18" t="str">
-        <f>_03_SOMD_search_eq[[#This Row],[ss_type]]&amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_authors]],5) &amp; "_" &amp; RIGHT(_03_SOMD_search_eq[[#This Row],[search_database_year]],2) &amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_title]],5) &amp; "_" &amp; LEFT(_03_SOMD_search_eq[[#This Row],[search_database_journal]],2)</f>
-        <v>_MFL A__Open _</v>
-      </c>
-      <c r="L10" s="12"/>
+      <c r="K6" s="17"/>
+      <c r="L6" s="18"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="G4">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
-  </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="G3" r:id="rId1" tooltip="Persistent link using digital object identifier" display="https://doi.org/10.1016/j.ecolecon.2022.107595" xr:uid="{B451EF4F-68A5-46B5-A414-4186B98EB6BC}"/>
-    <hyperlink ref="C8" r:id="rId2" xr:uid="{6D84DCF7-A9FB-4607-A8A6-5A52712B10AA}"/>
-    <hyperlink ref="C7" r:id="rId3" xr:uid="{20217A07-CD2E-47CF-A00F-B61A5353EDEB}"/>
-    <hyperlink ref="C9" r:id="rId4" xr:uid="{64AFC39D-2E46-4031-815F-D5FF42AAB727}"/>
-    <hyperlink ref="C10" r:id="rId5" xr:uid="{CC31478A-1163-4778-8684-72AAEC1CBC75}"/>
+    <hyperlink ref="G4" r:id="rId1" xr:uid="{6D84DCF7-A9FB-4607-A8A6-5A52712B10AA}"/>
+    <hyperlink ref="G3" r:id="rId2" xr:uid="{20217A07-CD2E-47CF-A00F-B61A5353EDEB}"/>
+    <hyperlink ref="G5" r:id="rId3" xr:uid="{64AFC39D-2E46-4031-815F-D5FF42AAB727}"/>
+    <hyperlink ref="G6" r:id="rId4" xr:uid="{CC31478A-1163-4778-8684-72AAEC1CBC75}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId6"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1656,7 +1513,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="B1" s="2">
         <v>3</v>
@@ -1664,31 +1521,31 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="1" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="1" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="B5">
         <v>11</v>
@@ -1696,42 +1553,42 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="1" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>46</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="B8" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="D8" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="E8" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="F8" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1739,19 +1596,19 @@
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="C9" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="D9" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="E9" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="F9" t="s">
-        <v>56</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1759,19 +1616,19 @@
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="C10" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="D10" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="E10" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="F10" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1779,19 +1636,19 @@
         <v>4</v>
       </c>
       <c r="B11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" t="s">
+        <v>45</v>
+      </c>
+      <c r="D11" t="s">
+        <v>46</v>
+      </c>
+      <c r="E11" t="s">
+        <v>47</v>
+      </c>
+      <c r="F11" t="s">
         <v>48</v>
-      </c>
-      <c r="C11" t="s">
-        <v>61</v>
-      </c>
-      <c r="D11" t="s">
-        <v>62</v>
-      </c>
-      <c r="E11" t="s">
-        <v>63</v>
-      </c>
-      <c r="F11" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1799,19 +1656,19 @@
         <v>5</v>
       </c>
       <c r="B12" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="C12" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="D12" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="E12" t="s">
-        <v>67</v>
+        <v>51</v>
       </c>
       <c r="F12" t="s">
-        <v>68</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1819,19 +1676,19 @@
         <v>6</v>
       </c>
       <c r="B13" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="C13" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="D13" t="s">
-        <v>70</v>
+        <v>54</v>
       </c>
       <c r="E13" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="F13" t="s">
-        <v>71</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -1839,19 +1696,19 @@
         <v>7</v>
       </c>
       <c r="B14" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="C14" t="s">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="D14" t="s">
-        <v>73</v>
+        <v>57</v>
       </c>
       <c r="E14" t="s">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="F14" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -1859,79 +1716,79 @@
         <v>8</v>
       </c>
       <c r="B15" t="s">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="C15" t="s">
-        <v>77</v>
+        <v>61</v>
       </c>
       <c r="D15" t="s">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="E15" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="F15" t="s">
-        <v>80</v>
+        <v>64</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>9</v>
+        <v>113</v>
       </c>
       <c r="B16" t="s">
-        <v>81</v>
+        <v>65</v>
       </c>
       <c r="C16" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="D16" t="s">
-        <v>83</v>
+        <v>67</v>
       </c>
       <c r="E16" t="s">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="F16" t="s">
-        <v>85</v>
+        <v>69</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B17" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="C17" t="s">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="D17" t="s">
-        <v>87</v>
+        <v>71</v>
       </c>
       <c r="E17" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="F17" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>81</v>
+        <v>65</v>
       </c>
       <c r="C18" t="s">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="D18" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="E18" t="s">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="F18" t="s">
-        <v>91</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1952,71 +1809,71 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="5" t="s">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>94</v>
-      </c>
-      <c r="C2" s="8"/>
+        <v>78</v>
+      </c>
+      <c r="C2" s="6"/>
       <c r="D2" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>96</v>
-      </c>
-      <c r="C3" s="8"/>
+        <v>80</v>
+      </c>
+      <c r="C3" s="6"/>
       <c r="D3" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>98</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>99</v>
+        <v>82</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>83</v>
       </c>
       <c r="D4" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>101</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>102</v>
+        <v>85</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>86</v>
       </c>
       <c r="D5" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>104</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>105</v>
+        <v>88</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>89</v>
       </c>
       <c r="D6" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -2030,8 +1887,19 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005BE3C66ACF4393458051577D36AC6C25" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1b97c7f6381d52e0ece85968e631718a">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4b26243c-b736-4d9c-b036-479be2ad88a1" xmlns:ns3="432dd258-9dce-4cb3-b611-c68c0fbce7f3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="af6cb7be8893fd4f0d362fb6f7fa19cb" ns2:_="" ns3:_="">
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4b26243c-b736-4d9c-b036-479be2ad88a1">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="432dd258-9dce-4cb3-b611-c68c0fbce7f3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005BE3C66ACF4393458051577D36AC6C25" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4e0e0d96de7fb32b1678b66c28514d8e">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4b26243c-b736-4d9c-b036-479be2ad88a1" xmlns:ns3="432dd258-9dce-4cb3-b611-c68c0fbce7f3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ac451aab8c96dec805c937cbafca7133" ns2:_="" ns3:_="">
     <xsd:import namespace="4b26243c-b736-4d9c-b036-479be2ad88a1"/>
     <xsd:import namespace="432dd258-9dce-4cb3-b611-c68c0fbce7f3"/>
     <xsd:element name="properties">
@@ -2050,6 +1918,7 @@
                 <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -2107,6 +1976,11 @@
     <xsd:element name="MediaLengthInSeconds" ma:index="18" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="19" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
@@ -2224,17 +2098,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4b26243c-b736-4d9c-b036-479be2ad88a1">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="432dd258-9dce-4cb3-b611-c68c0fbce7f3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2245,10 +2108,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF49202F-C698-49A6-968F-C1FAD0B15B1C}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2A8A660-9284-4780-8ED0-4709E9BB833A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -2265,6 +2124,25 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1813E577-F865-4294-8301-50AECB8DA6EF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="4b26243c-b736-4d9c-b036-479be2ad88a1"/>
+    <ds:schemaRef ds:uri="432dd258-9dce-4cb3-b611-c68c0fbce7f3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AEDD599-11B4-46FE-854D-9923ECF7E41C}">
   <ds:schemaRefs>

</xml_diff>